<commit_message>
CI guard: one Python check whose exit code decides (tracked data/outputs/logs folders, DB files, .env files and key names in the tree and every commit), with tests on both OS; Excel cover shows the company's market and the beta table its index
</commit_message>
<xml_diff>
--- a/examples/035610_sotp_associate/035610_model_example.xlsx
+++ b/examples/035610_sotp_associate/035610_model_example.xlsx
@@ -358,7 +358,7 @@
     <t>기본</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml excel.default_scenario</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml excel.default_scenario</t>
   </si>
   <si>
     <t>🔸</t>
@@ -415,7 +415,7 @@
     <t>날짜</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.as_of</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.as_of</t>
   </si>
   <si>
     <t>2026-09-30</t>
@@ -427,7 +427,7 @@
     <t>할인 기준일(재무상태표일)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date</t>
   </si>
   <si>
     <t>순현금(6/30 재무상태표)과 시작점을 맞춘다. EV는 평가기준일로 이월</t>
@@ -436,7 +436,7 @@
     <t>현금흐름 시작일</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date + 1일</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date + 1일</t>
   </si>
   <si>
     <t>연 일수</t>
@@ -463,7 +463,7 @@
     <t>mid-year 할인(1=예, 0=기말)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.mid_year</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.mid_year</t>
   </si>
   <si>
     <t>명시 기간 마지막 연도(생성 시 고정)</t>
@@ -493,7 +493,7 @@
     <t>consolidated</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure (규칙 판정)</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure (규칙 판정)</t>
   </si>
   <si>
     <t>Bridge 시트의 구조 판단 규칙(valuation_rules.yaml) 결과와 같아야 한다</t>
@@ -619,7 +619,7 @@
     <t>Hamada 세율(언레버·리레버)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml beta.tax</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml beta.tax</t>
   </si>
   <si>
     <t>피어 대부분의 과세표준 구간 한계세율</t>
@@ -643,7 +643,7 @@
     <t>배</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (공개 모드 집계 입력)</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (공개 모드 집계 입력)</t>
   </si>
   <si>
     <t>자체 D/E 시점 평균(5개 시점, PC에서 계산한 집계값. 시점별 시가총액은 공개 모드에 표시하지 않음)</t>
@@ -742,7 +742,7 @@
     <t>중요 종속회사 상장 여부(1=예)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.listed_subsidiary (otrCprInvstmntSttus)</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.listed_subsidiary (otrCprInvstmntSttus)</t>
   </si>
   <si>
     <t>5. 기계적 예측 규칙 (P7-B 자동 초안 규칙)</t>
@@ -751,7 +751,7 @@
     <t>영구성장률 g(사람 값)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.human.g_terminal</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.human.g_terminal</t>
   </si>
   <si>
     <t>세 시나리오 같음. 2030년까지 출발 성장률에서 같은 폭으로 체감</t>
@@ -760,7 +760,7 @@
     <t>출발 성장률 → g 도달 연도</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.fade_to_terminal_by</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.fade_to_terminal_by</t>
   </si>
   <si>
     <t>2031~2032 = g</t>
@@ -769,7 +769,7 @@
     <t>D&amp;A 반기 ÷ 연간 하한</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.ebitda_rule</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.ebitda_rule</t>
   </si>
   <si>
     <t>반기 D&amp;A가 3개월 값으로 보이면 LTM = FY D&amp;A</t>
@@ -790,7 +790,7 @@
     <t>%p</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.segments</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.segments</t>
   </si>
   <si>
     <t>단일 부문(자동 초안: 부문 미수집)</t>
@@ -892,7 +892,7 @@
     <t>KOSDAQ</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.target.market</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.target.market</t>
   </si>
   <si>
     <t>C3 판정: CV q50 손실 개선</t>
@@ -991,7 +991,7 @@
     <t>곳</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml relative.n_warn</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml relative.n_warn</t>
   </si>
   <si>
     <t>N/M(분모 ≤ 0) 제외 후 표본 수</t>
@@ -1132,7 +1132,7 @@
     <t>정상 이익률 이동</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml scenarios.human · 상태 ⚠️(±2%p 사용자 지시)</t>
+    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml scenarios.human · 상태 ⚠️(±2%p 사용자 지시)</t>
   </si>
   <si>
     <t>표 5. 실제 차입(약정이자율·잔액, Kd 규칙의 '실제 가중' 계산용)</t>
@@ -3898,7 +3898,7 @@
     <t>v1</t>
   </si>
   <si>
-    <t>2026-10-23T08:57:41</t>
+    <t>2026-10-23T11:07:05</t>
   </si>
   <si>
     <t>그대로 유지한 판단 0건 · 남은 미처리 43건</t>
@@ -4099,7 +4099,7 @@
     <t>생성</t>
   </si>
   <si>
-    <t>src/excel/build.py ← C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_yzdskxji/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (P4, 엔진 형태 mechanical). 결과 확인: Checks 시트의 master check</t>
+    <t>src/excel/build.py ← C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (P4, 엔진 형태 mechanical). 결과 확인: Checks 시트의 master check</t>
   </si>
   <si>
     <t>현재 선택</t>

</xml_diff>

<commit_message>
Validation republished with the final re-check holdout (pass 8 / below 4 / not measured 1, as measured); check-cell formulas never show an error on N/M (fixed after the measurement, values unchanged); known issues with status; methodology adds listing checks, share-event window, candidate ranges and reconciliation tolerances; snapshots and examples rebuilt
</commit_message>
<xml_diff>
--- a/examples/035610_sotp_associate/035610_model_example.xlsx
+++ b/examples/035610_sotp_associate/035610_model_example.xlsx
@@ -82,7 +82,7 @@
     <definedName name="DiagLightPeer">Diagnostics!$B$21</definedName>
     <definedName name="DiagMistagTable">Diagnostics!$A$161:$D$161</definedName>
     <definedName name="DiagMktRatio">Diagnostics!$B$14</definedName>
-    <definedName name="DiagOtherTable">Diagnostics!$B$94:$D$117</definedName>
+    <definedName name="DiagOtherTable">Diagnostics!$B$93:$D$117</definedName>
     <definedName name="DiagPeerBasis">Diagnostics!$B$7</definedName>
     <definedName name="DiagPeerMed">Diagnostics!$B$9</definedName>
     <definedName name="DiagPeerN">Diagnostics!$B$11</definedName>
@@ -90,7 +90,7 @@
     <definedName name="DiagPrice">Diagnostics!$B$13</definedName>
     <definedName name="DiagQ25">Diagnostics!$B$8</definedName>
     <definedName name="DiagQ75">Diagnostics!$B$10</definedName>
-    <definedName name="DiagRankTable">Diagnostics!$A$72:$G$91</definedName>
+    <definedName name="DiagRankTable">Diagnostics!$A$72:$G$90</definedName>
     <definedName name="DiagRevTable">Diagnostics!$A$29:$D$33</definedName>
     <definedName name="DiagSensTable">Diagnostics!$A$64:$D$68</definedName>
     <definedName name="DiagSotpDisc30">Diagnostics!$B$149</definedName>
@@ -110,7 +110,7 @@
     <definedName name="DiagThMYLo">Diagnostics!$B$19</definedName>
     <definedName name="DiagThPHi">Diagnostics!$B$16</definedName>
     <definedName name="DiagThPLo">Diagnostics!$B$15</definedName>
-    <definedName name="DiagTop5Share">Diagnostics!$G$92</definedName>
+    <definedName name="DiagTop5Share">Diagnostics!$G$91</definedName>
     <definedName name="DiagTurnLtm">Diagnostics!$B$154</definedName>
     <definedName name="DiagTurnM0">Diagnostics!$B$155</definedName>
     <definedName name="DiagTurnPS">Diagnostics!$B$156</definedName>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2375" uniqueCount="1266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2376" uniqueCount="1266">
   <si>
     <t>Inputs — 입력값 (파란 글씨·노란 바탕 칸만 바꾼다)</t>
   </si>
@@ -358,7 +358,7 @@
     <t>기본</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml excel.default_scenario</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml excel.default_scenario</t>
   </si>
   <si>
     <t>🔸</t>
@@ -415,7 +415,7 @@
     <t>날짜</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.as_of</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.as_of</t>
   </si>
   <si>
     <t>2026-09-30</t>
@@ -427,7 +427,7 @@
     <t>할인 기준일(재무상태표일)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date</t>
   </si>
   <si>
     <t>순현금(6/30 재무상태표)과 시작점을 맞춘다. EV는 평가기준일로 이월</t>
@@ -436,7 +436,7 @@
     <t>현금흐름 시작일</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date + 1일</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.bs_date + 1일</t>
   </si>
   <si>
     <t>연 일수</t>
@@ -463,7 +463,7 @@
     <t>mid-year 할인(1=예, 0=기말)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.mid_year</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.mid_year</t>
   </si>
   <si>
     <t>명시 기간 마지막 연도(생성 시 고정)</t>
@@ -493,7 +493,7 @@
     <t>consolidated</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure (규칙 판정)</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure (규칙 판정)</t>
   </si>
   <si>
     <t>Bridge 시트의 구조 판단 규칙(valuation_rules.yaml) 결과와 같아야 한다</t>
@@ -619,7 +619,7 @@
     <t>Hamada 세율(언레버·리레버)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml beta.tax</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml beta.tax</t>
   </si>
   <si>
     <t>피어 대부분의 과세표준 구간 한계세율</t>
@@ -643,7 +643,7 @@
     <t>배</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (공개 모드 집계 입력)</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (공개 모드 집계 입력)</t>
   </si>
   <si>
     <t>자체 D/E 시점 평균(5개 시점, PC에서 계산한 집계값. 시점별 시가총액은 공개 모드에 표시하지 않음)</t>
@@ -742,7 +742,7 @@
     <t>중요 종속회사 상장 여부(1=예)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.listed_subsidiary (otrCprInvstmntSttus)</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.listed_subsidiary (otrCprInvstmntSttus)</t>
   </si>
   <si>
     <t>5. 기계적 예측 규칙 (P7-B 자동 초안 규칙)</t>
@@ -751,7 +751,7 @@
     <t>영구성장률 g(사람 값)</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.human.g_terminal</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml forecast.human.g_terminal</t>
   </si>
   <si>
     <t>세 시나리오 같음. 2030년까지 출발 성장률에서 같은 폭으로 체감</t>
@@ -760,7 +760,7 @@
     <t>출발 성장률 → g 도달 연도</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.fade_to_terminal_by</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.fade_to_terminal_by</t>
   </si>
   <si>
     <t>2031~2032 = g</t>
@@ -769,7 +769,7 @@
     <t>D&amp;A 반기 ÷ 연간 하한</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.ebitda_rule</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml params.ebitda_rule</t>
   </si>
   <si>
     <t>반기 D&amp;A가 3개월 값으로 보이면 LTM = FY D&amp;A</t>
@@ -790,7 +790,7 @@
     <t>%p</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.segments</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml structure.segments</t>
   </si>
   <si>
     <t>단일 부문(자동 초안: 부문 미수집)</t>
@@ -892,7 +892,7 @@
     <t>KOSDAQ</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.target.market</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml meta.target.market</t>
   </si>
   <si>
     <t>C3 판정: CV q50 손실 개선</t>
@@ -991,7 +991,7 @@
     <t>곳</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml relative.n_warn</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml relative.n_warn</t>
   </si>
   <si>
     <t>N/M(분모 ≤ 0) 제외 후 표본 수</t>
@@ -1132,7 +1132,7 @@
     <t>정상 이익률 이동</t>
   </si>
   <si>
-    <t>C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml scenarios.human · 상태 ⚠️(±2%p 사용자 지시)</t>
+    <t>공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml scenarios.human · 상태 ⚠️(±2%p 사용자 지시)</t>
   </si>
   <si>
     <t>표 5. 실제 차입(약정이자율·잔액, Kd 규칙의 '실제 가중' 계산용)</t>
@@ -2785,7 +2785,7 @@
     <t>Checks — 모델 점검</t>
   </si>
   <si>
-    <t>ERR가 하나라도 있으면 master check = ERR. WARN은 주의 표시, INFO는 엔진 값 대조(입력을 바꾸면 달라지는 것이 정상)</t>
+    <t>ERR(또는 이 표 안 수식 오류)가 하나라도 있으면 master check = ERR. WARN은 주의 표시, INFO는 엔진 값 대조(입력을 바꾸면 달라지는 것이 정상). N/M = 양쪽 모두 숫자가 아님(일치), 한쪽만 N/M이면 DIFF</t>
   </si>
   <si>
     <t>#</t>
@@ -3496,7 +3496,7 @@
     <t>LTM 영업이익률 -101.4% vs 5년 중앙값 1.5%</t>
   </si>
   <si>
-    <t>LTM 이익률 출발 → 주당 7,656원</t>
+    <t>후보 없음(범위 밖: -101.40%)</t>
   </si>
   <si>
     <t>3 ★</t>
@@ -3547,202 +3547,202 @@
     <t>기본 경로 v1(3년 평균 이익률 -5.08%, 매출 CAGR 0.81%)</t>
   </si>
   <si>
+    <t>이익률 수렴</t>
+  </si>
+  <si>
+    <t>피어 쪽 수렴 비율</t>
+  </si>
+  <si>
+    <t>수렴 비율 0%(기본 50%, 피어 이익률 중앙값 12.4% 쪽)</t>
+  </si>
+  <si>
+    <t>시나리오 폭</t>
+  </si>
+  <si>
+    <t>±2%p(성장·이익률) 기본값, g 2%</t>
+  </si>
+  <si>
+    <t>낙관(+2%p)</t>
+  </si>
+  <si>
+    <t>할인율</t>
+  </si>
+  <si>
+    <t>SRP 열</t>
+  </si>
+  <si>
+    <t>SRP 2%</t>
+  </si>
+  <si>
+    <t>MRP</t>
+  </si>
+  <si>
+    <t>MRP 7%(기본 8%, 한공회 가이던스 7~9%)</t>
+  </si>
+  <si>
+    <t>수렴 도달 연도</t>
+  </si>
+  <si>
+    <t>도달 연도 2030(기본 2032)</t>
+  </si>
+  <si>
     <t>재투자 비율</t>
   </si>
   <si>
+    <t>D&amp;A ÷ 매출(3년 평균)</t>
+  </si>
+  <si>
+    <t>D&amp;A ÷ 매출 5년 평균 2.92%(FY2021~2025, 기본 3년 평균 2.42%)</t>
+  </si>
+  <si>
+    <t>CAPEX ÷ 매출(3년 평균)</t>
+  </si>
+  <si>
+    <t>CAPEX ÷ 매출 5년 평균 0.84%(FY2021~2025, 기본 3년 평균 1.31%)</t>
+  </si>
+  <si>
+    <t>Rf 만기</t>
+  </si>
+  <si>
+    <t>Rf 국고채 10년</t>
+  </si>
+  <si>
+    <t>목표 D/E(자기 평균)</t>
+  </si>
+  <si>
+    <t>피어 D/E 중앙값 0.015배(기본 자기 평균 0.004배)</t>
+  </si>
+  <si>
+    <t>비영업·현금성 분류</t>
+  </si>
+  <si>
+    <t>고객 자금 성격 현금</t>
+  </si>
+  <si>
+    <t>영업용 현금 0억을 브리지에서 뺌</t>
+  </si>
+  <si>
+    <t>g 2%(사람 값 기본)</t>
+  </si>
+  <si>
+    <t>g 3%</t>
+  </si>
+  <si>
+    <t>Kd 근거</t>
+  </si>
+  <si>
+    <t>신용등급 자동 탐색 안 함</t>
+  </si>
+  <si>
+    <t>세전 Kd 4.70%(AA- 3년, 기본 10.51%)</t>
+  </si>
+  <si>
+    <t>상위 5 항목 주당 영향 비중(영향 값 있는 항목 기준, P7-B5)</t>
+  </si>
+  <si>
+    <t>계산할 수 없는 항목(원래 순서)</t>
+  </si>
+  <si>
+    <t>우선주 처리</t>
+  </si>
+  <si>
+    <t>주식의 총수 표에 우선주 없음 — 확인만</t>
+  </si>
+  <si>
+    <t>피어 유사성</t>
+  </si>
+  <si>
+    <t>자동: KSIC 71310(앞 2자리 71), 시가총액 대상의 (공개 비표시)배, FY2023~2025 영업이익 흑자 — 사업 유사성 사람 검토 | 사업 개요: 2단계 피어 카드의 공시 인용 참고</t>
+  </si>
+  <si>
+    <t>자동: KSIC 716(앞 2자리 71), 시가총액 대상의 (공개 비표시)배, FY2023~2025 영업이익 흑자 — 사업 유사성 사람 검토 | 사업 개요: 2단계 피어 카드의 공시 인용 참고</t>
+  </si>
+  <si>
+    <t>상장 종속회사 지분 할인(기본 0%)</t>
+  </si>
+  <si>
+    <t>지주회사 할인 30%·50% 민감도 — 평가 목적에 맞는 할인을 사람이 정함</t>
+  </si>
+  <si>
+    <t>비상장 종속회사 장부가</t>
+  </si>
+  <si>
+    <t>장부가(취득원가 기준일 수 있음) — 공정가치와 다를 수 있음(P/B 민감도 참고)</t>
+  </si>
+  <si>
+    <t>기준일 뒤 주요 공시</t>
+  </si>
+  <si>
+    <t>2026-07-01~기준일 공시 7건(제목만, 주요 단어 0건)</t>
+  </si>
+  <si>
+    <t>반기보고서 (2026.06); 임원ㆍ주요주주특정증권등소유상황보고서; 주식등의대량보유상황보고서(일반)</t>
+  </si>
+  <si>
+    <t>FY2022 세전이익 − 영업이익 = -110억(영업이익 -3억의 30% 초과): 영업외 손익 확인</t>
+  </si>
+  <si>
+    <t>FY2023 세전이익 − 영업이익 = 34억(영업이익 15억의 30% 초과): 영업외 손익 확인</t>
+  </si>
+  <si>
+    <t>FY2024 세전이익 − 영업이익 = -54억(영업이익 1억의 30% 초과): 영업외 손익 확인</t>
+  </si>
+  <si>
+    <t>FY2025 세전이익 − 영업이익 = -31억(영업이익 -18억의 30% 초과): 영업외 손익 확인</t>
+  </si>
+  <si>
+    <t>FY2021~2025 영업이익률 범위 -48.7%~41.4%(폭 5%p 초과): 일회성 손익 여부 확인</t>
+  </si>
+  <si>
+    <t>보고서 사람 작성 칸</t>
+  </si>
+  <si>
+    <t>평가방법 선택 근거·채택·가중치</t>
+  </si>
+  <si>
+    <t>보고서 초안의 [사람 작성 칸]</t>
+  </si>
+  <si>
+    <t>정상화 조정(비경상 손익)</t>
+  </si>
+  <si>
+    <t>우발채무·비영업자산 명세 확인</t>
+  </si>
+  <si>
+    <t>DLOM·경영권 프리미엄 조정 여부와 근거</t>
+  </si>
+  <si>
+    <t>주요 가정의 합리성</t>
+  </si>
+  <si>
+    <t>평가상 한계 보완</t>
+  </si>
+  <si>
+    <t>구조(추가)</t>
+  </si>
+  <si>
+    <t>상장 피투자회사 ㈜인피니트헬스케어 48.7%</t>
+  </si>
+  <si>
+    <t>사실상 지배(연결) 여부 확인 — 구조 규칙은 지분 &gt; 50%만 상장 종속회사로 봄</t>
+  </si>
+  <si>
+    <t>상장 피투자회사 키네마스터(주) 30.5%</t>
+  </si>
+  <si>
+    <t>블록 프리미엄 입력</t>
+  </si>
+  <si>
+    <t>지분 구간 25~50%, 인수자 전략적, 2015~2026</t>
+  </si>
+  <si>
+    <t>기본값 — 평가 목적에 맞는지 확인</t>
+  </si>
+  <si>
     <t>운전자본 회전일수(3년 평균)</t>
   </si>
   <si>
-    <t>회전일수 5년 평균 DSO 432·DIO 4·DPO 5831일(FY2021~2025, 기본 DSO 120·DIO 2·DPO 4890일)</t>
-  </si>
-  <si>
-    <t>이익률 수렴</t>
-  </si>
-  <si>
-    <t>피어 쪽 수렴 비율</t>
-  </si>
-  <si>
-    <t>수렴 비율 0%(기본 50%, 피어 이익률 중앙값 12.4% 쪽)</t>
-  </si>
-  <si>
-    <t>시나리오 폭</t>
-  </si>
-  <si>
-    <t>±2%p(성장·이익률) 기본값, g 2%</t>
-  </si>
-  <si>
-    <t>낙관(+2%p)</t>
-  </si>
-  <si>
-    <t>할인율</t>
-  </si>
-  <si>
-    <t>SRP 열</t>
-  </si>
-  <si>
-    <t>SRP 2%</t>
-  </si>
-  <si>
-    <t>MRP</t>
-  </si>
-  <si>
-    <t>MRP 7%(기본 8%, 한공회 가이던스 7~9%)</t>
-  </si>
-  <si>
-    <t>수렴 도달 연도</t>
-  </si>
-  <si>
-    <t>도달 연도 2030(기본 2032)</t>
-  </si>
-  <si>
-    <t>D&amp;A ÷ 매출(3년 평균)</t>
-  </si>
-  <si>
-    <t>D&amp;A ÷ 매출 5년 평균 2.92%(FY2021~2025, 기본 3년 평균 2.42%)</t>
-  </si>
-  <si>
-    <t>CAPEX ÷ 매출(3년 평균)</t>
-  </si>
-  <si>
-    <t>CAPEX ÷ 매출 5년 평균 0.84%(FY2021~2025, 기본 3년 평균 1.31%)</t>
-  </si>
-  <si>
-    <t>Rf 만기</t>
-  </si>
-  <si>
-    <t>Rf 국고채 10년</t>
-  </si>
-  <si>
-    <t>목표 D/E(자기 평균)</t>
-  </si>
-  <si>
-    <t>피어 D/E 중앙값 0.015배(기본 자기 평균 0.004배)</t>
-  </si>
-  <si>
-    <t>비영업·현금성 분류</t>
-  </si>
-  <si>
-    <t>고객 자금 성격 현금</t>
-  </si>
-  <si>
-    <t>영업용 현금 0억을 브리지에서 뺌</t>
-  </si>
-  <si>
-    <t>g 2%(사람 값 기본)</t>
-  </si>
-  <si>
-    <t>g 3%</t>
-  </si>
-  <si>
-    <t>Kd 근거</t>
-  </si>
-  <si>
-    <t>신용등급 자동 탐색 안 함</t>
-  </si>
-  <si>
-    <t>세전 Kd 4.70%(AA- 3년, 기본 10.51%)</t>
-  </si>
-  <si>
-    <t>상위 5 항목 주당 영향 비중(영향 값 있는 항목 기준, P7-B5)</t>
-  </si>
-  <si>
-    <t>계산할 수 없는 항목(원래 순서)</t>
-  </si>
-  <si>
-    <t>우선주 처리</t>
-  </si>
-  <si>
-    <t>주식의 총수 표에 우선주 없음 — 확인만</t>
-  </si>
-  <si>
-    <t>피어 유사성</t>
-  </si>
-  <si>
-    <t>자동: KSIC 71310(앞 2자리 71), 시가총액 대상의 (공개 비표시)배, FY2023~2025 영업이익 흑자 — 사업 유사성 사람 검토 | 사업 개요: 2단계 피어 카드의 공시 인용 참고</t>
-  </si>
-  <si>
-    <t>자동: KSIC 716(앞 2자리 71), 시가총액 대상의 (공개 비표시)배, FY2023~2025 영업이익 흑자 — 사업 유사성 사람 검토 | 사업 개요: 2단계 피어 카드의 공시 인용 참고</t>
-  </si>
-  <si>
-    <t>상장 종속회사 지분 할인(기본 0%)</t>
-  </si>
-  <si>
-    <t>지주회사 할인 30%·50% 민감도 — 평가 목적에 맞는 할인을 사람이 정함</t>
-  </si>
-  <si>
-    <t>비상장 종속회사 장부가</t>
-  </si>
-  <si>
-    <t>장부가(취득원가 기준일 수 있음) — 공정가치와 다를 수 있음(P/B 민감도 참고)</t>
-  </si>
-  <si>
-    <t>기준일 뒤 주요 공시</t>
-  </si>
-  <si>
-    <t>2026-07-01~기준일 공시 7건(제목만, 주요 단어 0건)</t>
-  </si>
-  <si>
-    <t>반기보고서 (2026.06); 임원ㆍ주요주주특정증권등소유상황보고서; 주식등의대량보유상황보고서(일반)</t>
-  </si>
-  <si>
-    <t>FY2022 세전이익 − 영업이익 = -110억(영업이익 -3억의 30% 초과): 영업외 손익 확인</t>
-  </si>
-  <si>
-    <t>FY2023 세전이익 − 영업이익 = 34억(영업이익 15억의 30% 초과): 영업외 손익 확인</t>
-  </si>
-  <si>
-    <t>FY2024 세전이익 − 영업이익 = -54억(영업이익 1억의 30% 초과): 영업외 손익 확인</t>
-  </si>
-  <si>
-    <t>FY2025 세전이익 − 영업이익 = -31억(영업이익 -18억의 30% 초과): 영업외 손익 확인</t>
-  </si>
-  <si>
-    <t>FY2021~2025 영업이익률 범위 -48.7%~41.4%(폭 5%p 초과): 일회성 손익 여부 확인</t>
-  </si>
-  <si>
-    <t>보고서 사람 작성 칸</t>
-  </si>
-  <si>
-    <t>평가방법 선택 근거·채택·가중치</t>
-  </si>
-  <si>
-    <t>보고서 초안의 [사람 작성 칸]</t>
-  </si>
-  <si>
-    <t>정상화 조정(비경상 손익)</t>
-  </si>
-  <si>
-    <t>우발채무·비영업자산 명세 확인</t>
-  </si>
-  <si>
-    <t>DLOM·경영권 프리미엄 조정 여부와 근거</t>
-  </si>
-  <si>
-    <t>주요 가정의 합리성</t>
-  </si>
-  <si>
-    <t>평가상 한계 보완</t>
-  </si>
-  <si>
-    <t>구조(추가)</t>
-  </si>
-  <si>
-    <t>상장 피투자회사 ㈜인피니트헬스케어 48.7%</t>
-  </si>
-  <si>
-    <t>사실상 지배(연결) 여부 확인 — 구조 규칙은 지분 &gt; 50%만 상장 종속회사로 봄</t>
-  </si>
-  <si>
-    <t>상장 피투자회사 키네마스터(주) 30.5%</t>
-  </si>
-  <si>
-    <t>블록 프리미엄 입력</t>
-  </si>
-  <si>
-    <t>지분 구간 25~50%, 인수자 전략적, 2015~2026</t>
-  </si>
-  <si>
-    <t>기본값 — 평가 목적에 맞는지 확인</t>
+    <t>자동 진단(config/p7b2.yaml ranking)</t>
   </si>
   <si>
     <t>H. 대표값 판정(유효성 가드, 사전 고정 91a84dd)</t>
@@ -3898,7 +3898,7 @@
     <t>v1</t>
   </si>
   <si>
-    <t>2026-10-23T11:07:05</t>
+    <t>2026-10-24T02:02:27</t>
   </si>
   <si>
     <t>그대로 유지한 판단 0건 · 남은 미처리 43건</t>
@@ -4099,7 +4099,7 @@
     <t>생성</t>
   </si>
   <si>
-    <t>src/excel/build.py ← C:/Users/Mevius/AppData/Local/Temp/kvi_p7d_dta74qf4/ws/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (P4, 엔진 형태 mechanical). 결과 확인: Checks 시트의 master check</t>
+    <t>src/excel/build.py ← 공개 배포 작업 공간/sessions/035610_20260930_001/v1_public/valuation_035610_035610_20260930_001v1p.yaml (P4, 엔진 형태 mechanical). 결과 확인: Checks 시트의 master check</t>
   </si>
   <si>
     <t>현재 선택</t>
@@ -6019,7 +6019,7 @@
     </row>
     <row r="22" spans="2:3">
       <c r="B22" s="7" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="C22" s="8"/>
     </row>
@@ -15747,11 +15747,11 @@
         <v>967</v>
       </c>
       <c r="C3" s="3" t="str">
-        <f>IF(COUNTIF($C$6:$C$74,"ERR")=0,"OK","ERR")</f>
+        <f>IF(AND(COUNTIF($C$6:$C$74,"ERR")=0,SUMPRODUCT(ISERROR($C$6:$E$74)*1)=0),"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D3" s="7" t="str">
-        <f>"ERR "&amp;COUNTIF($C$6:$C$74,"ERR")&amp;" / WARN "&amp;COUNTIF($C$6:$C$74,"WARN")&amp;" / INFO 차이 "&amp;COUNTIF($C$6:$C$74,"DIFF")</f>
+        <f>"ERR "&amp;COUNTIF($C$6:$C$74,"ERR")&amp;" / WARN "&amp;COUNTIF($C$6:$C$74,"WARN")&amp;" / INFO 차이 "&amp;COUNTIF($C$6:$C$74,"DIFF")&amp;IF(SUMPRODUCT(ISERROR($C$6:$E$74)*1)&gt;0," / 수식 오류 "&amp;SUMPRODUCT(ISERROR($C$6:$E$74)*1),"")</f>
         <v>ERR 0 / WARN 3 / INFO 차이 0</v>
       </c>
     </row>
@@ -16184,11 +16184,11 @@
         <v>857</v>
       </c>
       <c r="C25" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Cover!$A$1:$B$2))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Cover!$A$1:$B$2)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D25" s="5">
-        <f>SUMPRODUCT(--ISERROR(Cover!$A$1:$B$2))</f>
+        <f>SUMPRODUCT(ISERROR(Cover!$A$1:$B$2)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E25" s="7" t="s">
@@ -16209,11 +16209,11 @@
         <v>861</v>
       </c>
       <c r="C26" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Forecast!$A$1:$R$95))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Forecast!$A$1:$R$95)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D26" s="5">
-        <f>SUMPRODUCT(--ISERROR(Forecast!$A$1:$R$95))</f>
+        <f>SUMPRODUCT(ISERROR(Forecast!$A$1:$R$95)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E26" s="7" t="s">
@@ -16234,11 +16234,11 @@
         <v>863</v>
       </c>
       <c r="C27" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(WACC!$A$1:$E$33))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(WACC!$A$1:$E$33)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D27" s="5">
-        <f>SUMPRODUCT(--ISERROR(WACC!$A$1:$E$33))</f>
+        <f>SUMPRODUCT(ISERROR(WACC!$A$1:$E$33)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E27" s="7" t="s">
@@ -16259,11 +16259,11 @@
         <v>865</v>
       </c>
       <c r="C28" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(DCF!$A$1:$R$59))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(DCF!$A$1:$R$59)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D28" s="5">
-        <f>SUMPRODUCT(--ISERROR(DCF!$A$1:$R$59))</f>
+        <f>SUMPRODUCT(ISERROR(DCF!$A$1:$R$59)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E28" s="7" t="s">
@@ -16284,11 +16284,11 @@
         <v>867</v>
       </c>
       <c r="C29" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Bridge!$A$1:$D$37))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Bridge!$A$1:$D$37)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D29" s="5">
-        <f>SUMPRODUCT(--ISERROR(Bridge!$A$1:$D$37))</f>
+        <f>SUMPRODUCT(ISERROR(Bridge!$A$1:$D$37)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E29" s="7" t="s">
@@ -16309,11 +16309,11 @@
         <v>869</v>
       </c>
       <c r="C30" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Peers!$A$1:$N$20))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Peers!$A$1:$N$20)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D30" s="5">
-        <f>SUMPRODUCT(--ISERROR(Peers!$A$1:$N$20))</f>
+        <f>SUMPRODUCT(ISERROR(Peers!$A$1:$N$20)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E30" s="7" t="s">
@@ -16334,11 +16334,11 @@
         <v>871</v>
       </c>
       <c r="C31" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Premium!$A$1:$F$33))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Premium!$A$1:$F$33)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D31" s="5">
-        <f>SUMPRODUCT(--ISERROR(Premium!$A$1:$F$33))</f>
+        <f>SUMPRODUCT(ISERROR(Premium!$A$1:$F$33)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E31" s="7" t="s">
@@ -16359,11 +16359,11 @@
         <v>873</v>
       </c>
       <c r="C32" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Scenarios!$A$1:$T$138))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Scenarios!$A$1:$T$138)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D32" s="5">
-        <f>SUMPRODUCT(--ISERROR(Scenarios!$A$1:$T$138))</f>
+        <f>SUMPRODUCT(ISERROR(Scenarios!$A$1:$T$138)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E32" s="7" t="s">
@@ -16384,11 +16384,11 @@
         <v>875</v>
       </c>
       <c r="C33" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Scen_Calc!$A$1:$R$220))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Scen_Calc!$A$1:$R$220)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D33" s="5">
-        <f>SUMPRODUCT(--ISERROR(Scen_Calc!$A$1:$R$220))</f>
+        <f>SUMPRODUCT(ISERROR(Scen_Calc!$A$1:$R$220)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E33" s="7" t="s">
@@ -16409,11 +16409,11 @@
         <v>877</v>
       </c>
       <c r="C34" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Football!$A$1:$H$15))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Football!$A$1:$H$15)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D34" s="5">
-        <f>SUMPRODUCT(--ISERROR(Football!$A$1:$H$15))</f>
+        <f>SUMPRODUCT(ISERROR(Football!$A$1:$H$15)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E34" s="7" t="s">
@@ -16434,11 +16434,11 @@
         <v>879</v>
       </c>
       <c r="C35" s="6" t="str">
-        <f>IF(SUMPRODUCT(--ISERROR(Convergence!$A$1:$G$17))=0,"OK","ERR")</f>
+        <f>IF(SUMPRODUCT(ISERROR(Convergence!$A$1:$G$17)*1)=0,"OK","ERR")</f>
         <v>OK</v>
       </c>
       <c r="D35" s="5">
-        <f>SUMPRODUCT(--ISERROR(Convergence!$A$1:$G$17))</f>
+        <f>SUMPRODUCT(ISERROR(Convergence!$A$1:$G$17)*1)</f>
         <v>0.0</v>
       </c>
       <c r="E35" s="7" t="s">
@@ -16619,7 +16619,7 @@
         <v>895</v>
       </c>
       <c r="C43" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(PerShare)),NOT(ISNUMBER(INDEX(Scenarios!$B$32:$D$34,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(PerShare-INDEX(Scenarios!$B$32:$D$34,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1,"OK","DIFF")))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(PerShare),ISNUMBER(INDEX(Scenarios!$B$32:$D$34,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(PerShare-INDEX(Scenarios!$B$32:$D$34,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(PerShare)),NOT(ISNUMBER(INDEX(Scenarios!$B$32:$D$34,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D43" s="5">
@@ -16645,7 +16645,7 @@
         <v>899</v>
       </c>
       <c r="C44" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(WACC)),NOT(ISNUMBER(INDEX(Scenarios!$B$37:$D$39,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(WACC-INDEX(Scenarios!$B$37:$D$39,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF")))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(WACC),ISNUMBER(INDEX(Scenarios!$B$37:$D$39,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(WACC-INDEX(Scenarios!$B$37:$D$39,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF"),IF(AND(NOT(ISNUMBER(WACC)),NOT(ISNUMBER(INDEX(Scenarios!$B$37:$D$39,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D44" s="5">
@@ -16671,7 +16671,7 @@
         <v>902</v>
       </c>
       <c r="C45" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(RONIC)),NOT(ISNUMBER(INDEX(Scenarios!$B$42:$D$44,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(RONIC-INDEX(Scenarios!$B$42:$D$44,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF")))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(RONIC),ISNUMBER(INDEX(Scenarios!$B$42:$D$44,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(RONIC-INDEX(Scenarios!$B$42:$D$44,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF"),IF(AND(NOT(ISNUMBER(RONIC)),NOT(ISNUMBER(INDEX(Scenarios!$B$42:$D$44,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D45" s="5">
@@ -16697,7 +16697,7 @@
         <v>904</v>
       </c>
       <c r="C46" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(TVShare)),NOT(ISNUMBER(INDEX(Scenarios!$B$47:$D$49,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(TVShare-INDEX(Scenarios!$B$47:$D$49,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF")))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(TVShare),ISNUMBER(INDEX(Scenarios!$B$47:$D$49,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(TVShare-INDEX(Scenarios!$B$47:$D$49,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF"),IF(AND(NOT(ISNUMBER(TVShare)),NOT(ISNUMBER(INDEX(Scenarios!$B$47:$D$49,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D46" s="5">
@@ -16723,7 +16723,7 @@
         <v>906</v>
       </c>
       <c r="C47" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(ImpliedMultiple)),NOT(ISNUMBER(INDEX(Scenarios!$B$52:$D$54,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(ImpliedMultiple-INDEX(Scenarios!$B$52:$D$54,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=0.0001,"OK","DIFF")))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(ImpliedMultiple),ISNUMBER(INDEX(Scenarios!$B$52:$D$54,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(ImpliedMultiple-INDEX(Scenarios!$B$52:$D$54,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=0.0001,"OK","DIFF"),IF(AND(NOT(ISNUMBER(ImpliedMultiple)),NOT(ISNUMBER(INDEX(Scenarios!$B$52:$D$54,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D47" s="5">
@@ -16749,8 +16749,8 @@
         <v>909</v>
       </c>
       <c r="C48" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(PerShareExit)),NOT(ISNUMBER(INDEX(Scenarios!$B$57:$D$59,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(PerShareExit-INDEX(Scenarios!$B$57:$D$59,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1,"OK","DIFF")))</f>
-        <v>N/A</v>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(PerShareExit),ISNUMBER(INDEX(Scenarios!$B$57:$D$59,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(PerShareExit-INDEX(Scenarios!$B$57:$D$59,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(PerShareExit)),NOT(ISNUMBER(INDEX(Scenarios!$B$57:$D$59,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
+        <v>N/M</v>
       </c>
       <c r="D48" s="5" t="str">
         <f>PerShareExit</f>
@@ -16775,7 +16775,7 @@
         <v>912</v>
       </c>
       <c r="C49" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(EV_930)),NOT(ISNUMBER(INDEX(Scenarios!$B$62:$D$64,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(EV_930-INDEX(Scenarios!$B$62:$D$64,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=0.01,"OK","DIFF")))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(EV_930),ISNUMBER(INDEX(Scenarios!$B$62:$D$64,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(EV_930-INDEX(Scenarios!$B$62:$D$64,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=0.01,"OK","DIFF"),IF(AND(NOT(ISNUMBER(EV_930)),NOT(ISNUMBER(INDEX(Scenarios!$B$62:$D$64,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D49" s="5">
@@ -16801,8 +16801,8 @@
         <v>915</v>
       </c>
       <c r="C50" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(ImpliedG_Exit)),NOT(ISNUMBER(INDEX(Scenarios!$B$67:$D$69,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(ImpliedG_Exit-INDEX(Scenarios!$B$67:$D$69,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF")))</f>
-        <v>N/A</v>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(ImpliedG_Exit),ISNUMBER(INDEX(Scenarios!$B$67:$D$69,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(ImpliedG_Exit-INDEX(Scenarios!$B$67:$D$69,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF"),IF(AND(NOT(ISNUMBER(ImpliedG_Exit)),NOT(ISNUMBER(INDEX(Scenarios!$B$67:$D$69,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
+        <v>N/M</v>
       </c>
       <c r="D50" s="5" t="str">
         <f>ImpliedG_Exit</f>
@@ -16827,8 +16827,8 @@
         <v>917</v>
       </c>
       <c r="C51" s="6" t="str">
-        <f>IF(AND(NOT(ISNUMBER(TVShare_Exit)),NOT(ISNUMBER(INDEX(Scenarios!$B$72:$D$74,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/A",IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(TVShare_Exit-INDEX(Scenarios!$B$72:$D$74,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF")))</f>
-        <v>N/A</v>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(TVShare_Exit),ISNUMBER(INDEX(Scenarios!$B$72:$D$74,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))),IF(ABS(TVShare_Exit-INDEX(Scenarios!$B$72:$D$74,ScenIdx,MATCH(SRP_Sel,SRP_List,0)))&lt;=1e-06,"OK","DIFF"),IF(AND(NOT(ISNUMBER(TVShare_Exit)),NOT(ISNUMBER(INDEX(Scenarios!$B$72:$D$74,ScenIdx,MATCH(SRP_Sel,SRP_List,0))))),"N/M","DIFF")))</f>
+        <v>N/M</v>
       </c>
       <c r="D51" s="5" t="str">
         <f>TVShare_Exit</f>
@@ -16922,7 +16922,7 @@
         <v>927</v>
       </c>
       <c r="C55" s="6" t="str">
-        <f>IF(ABS(BetaU-WACC!$E$6)&lt;1E-9,"OK","DIFF")</f>
+        <f>IF(AND(ISNUMBER(BetaU),ISNUMBER(WACC!$E$6)),IF(ABS(BetaU-WACC!$E$6)&lt;=1E-9,"OK","DIFF"),IF(AND(NOT(ISNUMBER(BetaU)),NOT(ISNUMBER(WACC!$E$6))),"N/M","DIFF"))</f>
         <v>OK</v>
       </c>
       <c r="D55" s="5">
@@ -17049,7 +17049,7 @@
         <v>937</v>
       </c>
       <c r="C60" s="6" t="str">
-        <f>IF(MAX(ABS(Block_q1-Premium!$E$23),ABS(Block_q2-Premium!$E$24),ABS(Block_q3-Premium!$E$25))&lt;=1,"OK","DIFF")</f>
+        <f>IF(AND(ISNUMBER(Block_q1),ISNUMBER(Premium!$E$23),ISNUMBER(Block_q2),ISNUMBER(Premium!$E$24),ISNUMBER(Block_q3),ISNUMBER(Premium!$E$25)),IF(MAX(ABS(Block_q1-Premium!$E$23),ABS(Block_q2-Premium!$E$24),ABS(Block_q3-Premium!$E$25))&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Block_q1)),NOT(ISNUMBER(Premium!$E$23)),NOT(ISNUMBER(Block_q2)),NOT(ISNUMBER(Premium!$E$24)),NOT(ISNUMBER(Block_q3)),NOT(ISNUMBER(Premium!$E$25))),"N/M","DIFF"))</f>
         <v>OK</v>
       </c>
       <c r="D60" s="5">
@@ -17120,7 +17120,7 @@
         <v>944</v>
       </c>
       <c r="C63" s="6" t="str">
-        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(ABS(Scenarios!$D$91-PerShare)&lt;=1,"OK","DIFF"),"N/A")</f>
+        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(AND(ISNUMBER(Scenarios!$D$91),ISNUMBER(PerShare)),IF(ABS(Scenarios!$D$91-PerShare)&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Scenarios!$D$91)),NOT(ISNUMBER(PerShare))),"N/M","DIFF")),"N/A")</f>
         <v>OK</v>
       </c>
       <c r="D63" s="5">
@@ -17168,7 +17168,7 @@
         <v>948</v>
       </c>
       <c r="C65" s="6" t="str">
-        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(ABS(Scenarios!$D$100-PerShare)&lt;=1,"OK","DIFF"),"N/A")</f>
+        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(AND(ISNUMBER(Scenarios!$D$100),ISNUMBER(PerShare)),IF(ABS(Scenarios!$D$100-PerShare)&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Scenarios!$D$100)),NOT(ISNUMBER(PerShare))),"N/M","DIFF")),"N/A")</f>
         <v>OK</v>
       </c>
       <c r="D65" s="5">
@@ -17216,7 +17216,7 @@
         <v>952</v>
       </c>
       <c r="C67" s="6" t="str">
-        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(ABS(Scenarios!$B$108-PerShare)&lt;=1,"OK","DIFF"),"N/A")</f>
+        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(AND(ISNUMBER(Scenarios!$B$108),ISNUMBER(PerShare)),IF(ABS(Scenarios!$B$108-PerShare)&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Scenarios!$B$108)),NOT(ISNUMBER(PerShare))),"N/M","DIFF")),"N/A")</f>
         <v>OK</v>
       </c>
       <c r="D67" s="5">
@@ -17264,7 +17264,7 @@
         <v>956</v>
       </c>
       <c r="C69" s="6" t="str">
-        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(ABS(Scenarios!$B$121-PerShare)&lt;=1,"OK","DIFF"),"N/A")</f>
+        <f>IF(AND(ScenSel="기본",SRP_Sel=SRP_1,RonicStart="normal",RfTenor=5),IF(AND(ISNUMBER(Scenarios!$B$121),ISNUMBER(PerShare)),IF(ABS(Scenarios!$B$121-PerShare)&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Scenarios!$B$121)),NOT(ISNUMBER(PerShare))),"N/M","DIFF")),"N/A")</f>
         <v>OK</v>
       </c>
       <c r="D69" s="5">
@@ -17310,7 +17310,7 @@
         <v>960</v>
       </c>
       <c r="C71" s="6" t="str">
-        <f>IF(ABS(Convergence!$B$13-Convergence!$B$8)&lt;=1,"OK","DIFF")</f>
+        <f>IF(AND(ISNUMBER(Convergence!$B$13),ISNUMBER(Convergence!$B$8)),IF(ABS(Convergence!$B$13-Convergence!$B$8)&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Convergence!$B$13)),NOT(ISNUMBER(Convergence!$B$8))),"N/M","DIFF"))</f>
         <v>OK</v>
       </c>
       <c r="D71" s="5">
@@ -17379,7 +17379,7 @@
         <v>966</v>
       </c>
       <c r="C74" s="6" t="str">
-        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(ABS(Scenarios!$K$91-INDEX(ScenGridPS,MATCH("기본",ScenNames,0),1))&lt;=1,"OK","DIFF"))</f>
+        <f>IF(RfTenor&lt;&gt;5,"N/A",IF(AND(ISNUMBER(Scenarios!$K$91),ISNUMBER(INDEX(ScenGridPS,MATCH("기본",ScenNames,0),1))),IF(ABS(Scenarios!$K$91-INDEX(ScenGridPS,MATCH("기본",ScenNames,0),1))&lt;=1,"OK","DIFF"),IF(AND(NOT(ISNUMBER(Scenarios!$K$91)),NOT(ISNUMBER(INDEX(ScenGridPS,MATCH("기본",ScenNames,0),1)))),"N/M","DIFF")))</f>
         <v>OK</v>
       </c>
       <c r="D74" s="5">
@@ -17399,27 +17399,33 @@
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"N/M"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"ERR"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
       <formula>"WARN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
       <formula>"DIFF"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C74">
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
+      <formula>"N/M"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
       <formula>"ERR"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="9" operator="equal">
       <formula>"WARN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="10" operator="equal">
       <formula>"DIFF"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18156,11 +18162,11 @@
       <c r="D73" s="4" t="s">
         <v>1058</v>
       </c>
-      <c r="F73" s="58">
-        <v>-1078.149368240279</v>
-      </c>
-      <c r="G73" s="18">
-        <v>-0.1234447104452636</v>
+      <c r="F73" s="58" t="s">
+        <v>695</v>
+      </c>
+      <c r="G73" s="18" t="s">
+        <v>695</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -18277,10 +18283,10 @@
         <v>1077</v>
       </c>
       <c r="F79" s="58">
-        <v>-118.7564841878429</v>
+        <v>-63.58306853807153</v>
       </c>
       <c r="G79" s="18">
-        <v>-0.01359724379191833</v>
+        <v>-0.00728006129402503</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -18297,10 +18303,10 @@
         <v>1080</v>
       </c>
       <c r="F80" s="58">
-        <v>-63.58306853807153</v>
+        <v>33.64209251420289</v>
       </c>
       <c r="G80" s="18">
-        <v>-0.00728006129402503</v>
+        <v>0.003851913743609423</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -18317,10 +18323,10 @@
         <v>1083</v>
       </c>
       <c r="F81" s="58">
-        <v>33.64209251420289</v>
+        <v>-17.37130866828738</v>
       </c>
       <c r="G81" s="18">
-        <v>0.003851913743609423</v>
+        <v>-0.001988960186576049</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -18328,19 +18334,19 @@
         <v>262</v>
       </c>
       <c r="B82" s="7" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C82" s="4" t="s">
         <v>1084</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="D82" s="4" t="s">
         <v>1085</v>
       </c>
-      <c r="D82" s="4" t="s">
-        <v>1086</v>
-      </c>
       <c r="F82" s="58">
-        <v>-17.37130866828738</v>
+        <v>7.106185666556485</v>
       </c>
       <c r="G82" s="18">
-        <v>-0.001988960186576049</v>
+        <v>0.0008136359003856028</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -18348,19 +18354,19 @@
         <v>839</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>1084</v>
+        <v>1075</v>
       </c>
       <c r="C83" s="4" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D83" s="4" t="s">
         <v>1087</v>
       </c>
-      <c r="D83" s="4" t="s">
-        <v>1088</v>
-      </c>
       <c r="F83" s="58">
-        <v>7.106185666556485</v>
+        <v>5.00898388254609</v>
       </c>
       <c r="G83" s="18">
-        <v>0.0008136359003856028</v>
+        <v>0.0005735128946141455</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -18368,7 +18374,7 @@
         <v>841</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>1078</v>
+        <v>1088</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>1089</v>
@@ -18377,10 +18383,10 @@
         <v>1090</v>
       </c>
       <c r="F84" s="58">
-        <v>5.00898388254609</v>
+        <v>3.713878922979347</v>
       </c>
       <c r="G84" s="18">
-        <v>0.0005735128946141455</v>
+        <v>0.0004252274515768023</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -18388,7 +18394,7 @@
         <v>843</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>1075</v>
+        <v>1088</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>1091</v>
@@ -18397,10 +18403,10 @@
         <v>1092</v>
       </c>
       <c r="F85" s="58">
-        <v>3.713878922979347</v>
+        <v>3.470542958279111</v>
       </c>
       <c r="G85" s="18">
-        <v>0.0004252274515768023</v>
+        <v>0.0003973662492348972</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -18408,7 +18414,7 @@
         <v>845</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>1075</v>
+        <v>1081</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>1093</v>
@@ -18417,10 +18423,10 @@
         <v>1094</v>
       </c>
       <c r="F86" s="58">
-        <v>3.470542958279111</v>
+        <v>-2.111033840203163</v>
       </c>
       <c r="G86" s="18">
-        <v>0.0003973662492348972</v>
+        <v>-0.0002417067326852576</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -18428,7 +18434,7 @@
         <v>847</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>1084</v>
+        <v>526</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>1095</v>
@@ -18437,10 +18443,10 @@
         <v>1096</v>
       </c>
       <c r="F87" s="58">
-        <v>-2.111033840203163</v>
+        <v>-0.435675711980366</v>
       </c>
       <c r="G87" s="18">
-        <v>-0.0002417067326852576</v>
+        <v>-4.988349824035181E-05</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -18448,19 +18454,19 @@
         <v>849</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>526</v>
+        <v>1097</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="F88" s="58">
-        <v>-0.435675711980366</v>
+        <v>-0.3102465051831901</v>
       </c>
       <c r="G88" s="18">
-        <v>-4.988349824035181E-05</v>
+        <v>-3.552224870428032E-05</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -18468,7 +18474,7 @@
         <v>851</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>1099</v>
+        <v>598</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>1100</v>
@@ -18477,10 +18483,10 @@
         <v>1101</v>
       </c>
       <c r="F89" s="58">
-        <v>-0.3102465051831901</v>
+        <v>0.286985117394579</v>
       </c>
       <c r="G89" s="18">
-        <v>-3.552224870428032E-05</v>
+        <v>3.285889299058468E-05</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -18488,51 +18494,42 @@
         <v>853</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>598</v>
+        <v>1102</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="F90" s="58">
-        <v>0.286985117394579</v>
+        <v>0.2332683255554002</v>
       </c>
       <c r="G90" s="18">
-        <v>3.285889299058468E-05</v>
+        <v>2.67084893359789E-05</v>
       </c>
     </row>
     <row r="91" spans="1:7">
-      <c r="A91" s="17" t="s">
-        <v>856</v>
-      </c>
-      <c r="B91" s="7" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C91" s="4" t="s">
+      <c r="A91" s="9" t="s">
         <v>1105</v>
       </c>
-      <c r="D91" s="4" t="s">
+      <c r="G91" s="18">
+        <v>0.9653924657015837</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
+      <c r="A92" s="11" t="s">
         <v>1106</v>
       </c>
-      <c r="F91" s="58">
-        <v>0.2332683255554002</v>
-      </c>
-      <c r="G91" s="18">
-        <v>2.67084893359789E-05</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7">
-      <c r="A92" s="9" t="s">
+    </row>
+    <row r="93" spans="1:7">
+      <c r="B93" s="7" t="s">
         <v>1107</v>
       </c>
-      <c r="G92" s="18">
-        <v>0.9166820597528649</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7">
-      <c r="A93" s="11" t="s">
+      <c r="C93" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D93" s="4" t="s">
         <v>1108</v>
       </c>
     </row>
@@ -18541,7 +18538,7 @@
         <v>1109</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>126</v>
+        <v>287</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>1110</v>
@@ -18549,68 +18546,68 @@
     </row>
     <row r="95" spans="1:7">
       <c r="B95" s="7" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="96" spans="1:7">
       <c r="B96" s="7" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="D96" s="4" t="s">
         <v>1111</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>1112</v>
       </c>
     </row>
     <row r="97" spans="2:4">
       <c r="B97" s="7" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="98" spans="2:4">
       <c r="B98" s="7" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="99" spans="2:4">
       <c r="B99" s="7" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="100" spans="2:4">
       <c r="B100" s="7" t="s">
-        <v>1111</v>
+        <v>1060</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>295</v>
+        <v>1112</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="101" spans="2:4">
@@ -18626,24 +18623,24 @@
     </row>
     <row r="102" spans="2:4">
       <c r="B102" s="7" t="s">
-        <v>1060</v>
+        <v>1116</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="103" spans="2:4">
       <c r="B103" s="7" t="s">
-        <v>1118</v>
+        <v>1069</v>
       </c>
       <c r="C103" s="4" t="s">
+        <v>1070</v>
+      </c>
+      <c r="D103" s="4" t="s">
         <v>1119</v>
-      </c>
-      <c r="D103" s="4" t="s">
-        <v>1120</v>
       </c>
     </row>
     <row r="104" spans="2:4">
@@ -18654,7 +18651,7 @@
         <v>1070</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="105" spans="2:4">
@@ -18665,7 +18662,7 @@
         <v>1070</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="106" spans="2:4">
@@ -18676,7 +18673,7 @@
         <v>1070</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="107" spans="2:4">
@@ -18687,111 +18684,111 @@
         <v>1070</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="108" spans="2:4">
       <c r="B108" s="7" t="s">
-        <v>1069</v>
+        <v>1124</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>1070</v>
+        <v>1125</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="109" spans="2:4">
       <c r="B109" s="7" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>1127</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="110" spans="2:4">
       <c r="B110" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>1128</v>
+      </c>
+      <c r="D110" s="4" t="s">
         <v>1126</v>
-      </c>
-      <c r="C110" s="4" t="s">
-        <v>1129</v>
-      </c>
-      <c r="D110" s="4" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="111" spans="2:4">
       <c r="B111" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>1129</v>
+      </c>
+      <c r="D111" s="4" t="s">
         <v>1126</v>
-      </c>
-      <c r="C111" s="4" t="s">
-        <v>1130</v>
-      </c>
-      <c r="D111" s="4" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="112" spans="2:4">
       <c r="B112" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D112" s="4" t="s">
         <v>1126</v>
-      </c>
-      <c r="C112" s="4" t="s">
-        <v>1131</v>
-      </c>
-      <c r="D112" s="4" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="B113" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>1131</v>
+      </c>
+      <c r="D113" s="4" t="s">
         <v>1126</v>
-      </c>
-      <c r="C113" s="4" t="s">
-        <v>1132</v>
-      </c>
-      <c r="D113" s="4" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="B114" s="7" t="s">
-        <v>1126</v>
+        <v>1132</v>
       </c>
       <c r="C114" s="4" t="s">
         <v>1133</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>1128</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="B115" s="7" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="C115" s="4" t="s">
         <v>1135</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="B116" s="7" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="C116" s="4" t="s">
         <v>1137</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="B117" s="7" t="s">
-        <v>1138</v>
+        <v>1088</v>
       </c>
       <c r="C117" s="4" t="s">
         <v>1139</v>
@@ -19017,7 +19014,7 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="7" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="B144" s="62">
         <v>29988</v>

</xml_diff>